<commit_message>
Incluida estructura para el reporte final
</commit_message>
<xml_diff>
--- a/docs/Casos de Regatas.xlsx
+++ b/docs/Casos de Regatas.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0b358109354d87fd/Diplomaturas/01. Inteligencia Artificial Aplicada/Materias/04. Procesamiento de Lenguaje Natural/99. DIIA-PLN-TP-Final/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0b358109354d87fd/Diplomaturas/01. Inteligencia Artificial Aplicada/Materias/05. Taller de Trabajo Final/Repositorio/DIIA_trabajo_final/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="578" documentId="11_2C447A9E1C490587C5EB8AD627D4F21B5C78B259" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{68382120-6E42-B04F-8967-EA922F9CED2A}"/>
+  <xr:revisionPtr revIDLastSave="582" documentId="11_2C447A9E1C490587C5EB8AD627D4F21B5C78B259" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0324D4F5-1AAE-3844-A7E1-FCF277E8EA75}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17460" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="80" yWindow="660" windowWidth="30160" windowHeight="17460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Casos de Regatas y sus Títulos" sheetId="1" r:id="rId1"/>
@@ -1939,7 +1939,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1973,24 +1973,107 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="5" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2000,94 +2083,14 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="5" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2352,10 +2355,10 @@
       <c r="B4" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="53" t="s">
         <v>23</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="53" t="s">
         <v>35</v>
       </c>
     </row>
@@ -2394,10 +2397,10 @@
       <c r="B7" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="53" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="53" t="s">
         <v>38</v>
       </c>
     </row>
@@ -2564,50 +2567,50 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="46" t="s">
         <v>59</v>
       </c>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18" t="s">
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
+      <c r="E2" s="46"/>
+      <c r="F2" s="46"/>
+      <c r="G2" s="46" t="s">
         <v>60</v>
       </c>
-      <c r="H2" s="25"/>
-      <c r="I2" s="25"/>
-      <c r="J2" s="25"/>
-      <c r="K2" s="25"/>
+      <c r="H2" s="47"/>
+      <c r="I2" s="47"/>
+      <c r="J2" s="47"/>
+      <c r="K2" s="47"/>
     </row>
     <row r="3" spans="1:11" ht="29" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="26" t="s">
+      <c r="A3" s="51" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="48" t="s">
         <v>50</v>
       </c>
-      <c r="C3" s="20"/>
-      <c r="D3" s="21" t="s">
+      <c r="C3" s="49"/>
+      <c r="D3" s="50" t="s">
         <v>51</v>
       </c>
-      <c r="E3" s="20"/>
-      <c r="F3" s="22" t="s">
+      <c r="E3" s="49"/>
+      <c r="F3" s="44" t="s">
         <v>52</v>
       </c>
-      <c r="G3" s="19" t="s">
+      <c r="G3" s="48" t="s">
         <v>50</v>
       </c>
-      <c r="H3" s="20"/>
-      <c r="I3" s="21" t="s">
+      <c r="H3" s="49"/>
+      <c r="I3" s="50" t="s">
         <v>51</v>
       </c>
-      <c r="J3" s="20"/>
-      <c r="K3" s="22" t="s">
+      <c r="J3" s="49"/>
+      <c r="K3" s="44" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A4" s="27"/>
+      <c r="A4" s="52"/>
       <c r="B4" s="6" t="s">
         <v>48</v>
       </c>
@@ -2620,7 +2623,7 @@
       <c r="E4" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="F4" s="23"/>
+      <c r="F4" s="45"/>
       <c r="G4" s="6" t="s">
         <v>48</v>
       </c>
@@ -2633,37 +2636,37 @@
       <c r="J4" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="K4" s="23"/>
+      <c r="K4" s="45"/>
     </row>
     <row r="5" spans="1:11" ht="28" x14ac:dyDescent="0.15">
-      <c r="A5" s="28">
+      <c r="A5" s="37">
         <v>1</v>
       </c>
-      <c r="B5" s="24" t="s">
-        <v>53</v>
-      </c>
-      <c r="C5" s="36" t="s">
-        <v>53</v>
-      </c>
-      <c r="D5" s="36" t="s">
-        <v>53</v>
-      </c>
-      <c r="E5" s="36" t="s">
+      <c r="B5" s="42" t="s">
+        <v>53</v>
+      </c>
+      <c r="C5" s="43" t="s">
+        <v>53</v>
+      </c>
+      <c r="D5" s="43" t="s">
+        <v>53</v>
+      </c>
+      <c r="E5" s="43" t="s">
         <v>53</v>
       </c>
       <c r="F5" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="G5" s="24" t="s">
-        <v>53</v>
-      </c>
-      <c r="H5" s="36" t="s">
-        <v>53</v>
-      </c>
-      <c r="I5" s="36" t="s">
-        <v>53</v>
-      </c>
-      <c r="J5" s="36" t="s">
+      <c r="G5" s="42" t="s">
+        <v>53</v>
+      </c>
+      <c r="H5" s="43" t="s">
+        <v>53</v>
+      </c>
+      <c r="I5" s="43" t="s">
+        <v>53</v>
+      </c>
+      <c r="J5" s="43" t="s">
         <v>53</v>
       </c>
       <c r="K5" s="8" t="s">
@@ -2671,85 +2674,85 @@
       </c>
     </row>
     <row r="6" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A6" s="29"/>
-      <c r="B6" s="13"/>
-      <c r="C6" s="17"/>
-      <c r="D6" s="17"/>
-      <c r="E6" s="17"/>
+      <c r="A6" s="38"/>
+      <c r="B6" s="32"/>
+      <c r="C6" s="40"/>
+      <c r="D6" s="40"/>
+      <c r="E6" s="40"/>
       <c r="F6" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="G6" s="13"/>
-      <c r="H6" s="17"/>
-      <c r="I6" s="17"/>
-      <c r="J6" s="17"/>
+      <c r="G6" s="32"/>
+      <c r="H6" s="40"/>
+      <c r="I6" s="40"/>
+      <c r="J6" s="40"/>
       <c r="K6" s="9" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="28" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A7" s="29"/>
-      <c r="B7" s="13"/>
-      <c r="C7" s="17"/>
-      <c r="D7" s="17"/>
-      <c r="E7" s="17"/>
+      <c r="A7" s="38"/>
+      <c r="B7" s="32"/>
+      <c r="C7" s="40"/>
+      <c r="D7" s="40"/>
+      <c r="E7" s="40"/>
       <c r="F7" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="G7" s="13"/>
-      <c r="H7" s="17"/>
-      <c r="I7" s="17"/>
-      <c r="J7" s="17"/>
+      <c r="G7" s="32"/>
+      <c r="H7" s="40"/>
+      <c r="I7" s="40"/>
+      <c r="J7" s="40"/>
       <c r="K7" s="9" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="28" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A8" s="30"/>
-      <c r="B8" s="13"/>
-      <c r="C8" s="17"/>
-      <c r="D8" s="17"/>
-      <c r="E8" s="17"/>
+      <c r="A8" s="39"/>
+      <c r="B8" s="32"/>
+      <c r="C8" s="40"/>
+      <c r="D8" s="40"/>
+      <c r="E8" s="40"/>
       <c r="F8" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="G8" s="13"/>
-      <c r="H8" s="17"/>
-      <c r="I8" s="17"/>
-      <c r="J8" s="17"/>
+      <c r="G8" s="32"/>
+      <c r="H8" s="40"/>
+      <c r="I8" s="40"/>
+      <c r="J8" s="40"/>
       <c r="K8" s="9" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A9" s="28">
+      <c r="A9" s="37">
         <v>2</v>
       </c>
-      <c r="B9" s="13" t="s">
-        <v>54</v>
-      </c>
-      <c r="C9" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="D9" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="E9" s="14" t="s">
+      <c r="B9" s="32" t="s">
+        <v>54</v>
+      </c>
+      <c r="C9" s="34" t="s">
+        <v>54</v>
+      </c>
+      <c r="D9" s="34" t="s">
+        <v>53</v>
+      </c>
+      <c r="E9" s="34" t="s">
         <v>54</v>
       </c>
       <c r="F9" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="G9" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="H9" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="I9" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="J9" s="14" t="s">
+      <c r="G9" s="32" t="s">
+        <v>53</v>
+      </c>
+      <c r="H9" s="34" t="s">
+        <v>53</v>
+      </c>
+      <c r="I9" s="34" t="s">
+        <v>53</v>
+      </c>
+      <c r="J9" s="34" t="s">
         <v>53</v>
       </c>
       <c r="K9" s="9" t="s">
@@ -2757,85 +2760,85 @@
       </c>
     </row>
     <row r="10" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A10" s="29"/>
-      <c r="B10" s="13"/>
-      <c r="C10" s="17"/>
-      <c r="D10" s="17"/>
-      <c r="E10" s="17"/>
+      <c r="A10" s="38"/>
+      <c r="B10" s="32"/>
+      <c r="C10" s="40"/>
+      <c r="D10" s="40"/>
+      <c r="E10" s="40"/>
       <c r="F10" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="G10" s="13"/>
-      <c r="H10" s="17"/>
-      <c r="I10" s="17"/>
-      <c r="J10" s="17"/>
+      <c r="G10" s="32"/>
+      <c r="H10" s="40"/>
+      <c r="I10" s="40"/>
+      <c r="J10" s="40"/>
       <c r="K10" s="9" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="11" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A11" s="29"/>
-      <c r="B11" s="13"/>
-      <c r="C11" s="17"/>
-      <c r="D11" s="17"/>
-      <c r="E11" s="17"/>
+      <c r="A11" s="38"/>
+      <c r="B11" s="32"/>
+      <c r="C11" s="40"/>
+      <c r="D11" s="40"/>
+      <c r="E11" s="40"/>
       <c r="F11" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="G11" s="13"/>
-      <c r="H11" s="17"/>
-      <c r="I11" s="17"/>
-      <c r="J11" s="17"/>
+      <c r="G11" s="32"/>
+      <c r="H11" s="40"/>
+      <c r="I11" s="40"/>
+      <c r="J11" s="40"/>
       <c r="K11" s="9" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="12" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A12" s="30"/>
-      <c r="B12" s="13"/>
-      <c r="C12" s="17"/>
-      <c r="D12" s="17"/>
-      <c r="E12" s="17"/>
+      <c r="A12" s="39"/>
+      <c r="B12" s="32"/>
+      <c r="C12" s="40"/>
+      <c r="D12" s="40"/>
+      <c r="E12" s="40"/>
       <c r="F12" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="G12" s="13"/>
-      <c r="H12" s="17"/>
-      <c r="I12" s="17"/>
-      <c r="J12" s="17"/>
+      <c r="G12" s="32"/>
+      <c r="H12" s="40"/>
+      <c r="I12" s="40"/>
+      <c r="J12" s="40"/>
       <c r="K12" s="9" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A13" s="28">
+      <c r="A13" s="37">
         <v>3</v>
       </c>
-      <c r="B13" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="C13" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="D13" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="E13" s="14" t="s">
+      <c r="B13" s="32" t="s">
+        <v>53</v>
+      </c>
+      <c r="C13" s="34" t="s">
+        <v>53</v>
+      </c>
+      <c r="D13" s="34" t="s">
+        <v>53</v>
+      </c>
+      <c r="E13" s="34" t="s">
         <v>53</v>
       </c>
       <c r="F13" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="G13" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="H13" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="I13" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="J13" s="14" t="s">
+      <c r="G13" s="32" t="s">
+        <v>53</v>
+      </c>
+      <c r="H13" s="34" t="s">
+        <v>53</v>
+      </c>
+      <c r="I13" s="34" t="s">
+        <v>53</v>
+      </c>
+      <c r="J13" s="34" t="s">
         <v>53</v>
       </c>
       <c r="K13" s="9" t="s">
@@ -2843,85 +2846,85 @@
       </c>
     </row>
     <row r="14" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A14" s="29"/>
-      <c r="B14" s="13"/>
-      <c r="C14" s="17"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="17"/>
+      <c r="A14" s="38"/>
+      <c r="B14" s="32"/>
+      <c r="C14" s="40"/>
+      <c r="D14" s="40"/>
+      <c r="E14" s="40"/>
       <c r="F14" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="G14" s="13"/>
-      <c r="H14" s="17"/>
-      <c r="I14" s="17"/>
-      <c r="J14" s="17"/>
+      <c r="G14" s="32"/>
+      <c r="H14" s="40"/>
+      <c r="I14" s="40"/>
+      <c r="J14" s="40"/>
       <c r="K14" s="9" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="15" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A15" s="29"/>
-      <c r="B15" s="13"/>
-      <c r="C15" s="17"/>
-      <c r="D15" s="17"/>
-      <c r="E15" s="17"/>
+      <c r="A15" s="38"/>
+      <c r="B15" s="32"/>
+      <c r="C15" s="40"/>
+      <c r="D15" s="40"/>
+      <c r="E15" s="40"/>
       <c r="F15" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="G15" s="13"/>
-      <c r="H15" s="17"/>
-      <c r="I15" s="17"/>
-      <c r="J15" s="17"/>
+      <c r="G15" s="32"/>
+      <c r="H15" s="40"/>
+      <c r="I15" s="40"/>
+      <c r="J15" s="40"/>
       <c r="K15" s="9" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="16" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A16" s="30"/>
-      <c r="B16" s="13"/>
-      <c r="C16" s="17"/>
-      <c r="D16" s="17"/>
-      <c r="E16" s="17"/>
+      <c r="A16" s="39"/>
+      <c r="B16" s="32"/>
+      <c r="C16" s="40"/>
+      <c r="D16" s="40"/>
+      <c r="E16" s="40"/>
       <c r="F16" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="G16" s="13"/>
-      <c r="H16" s="17"/>
-      <c r="I16" s="17"/>
-      <c r="J16" s="17"/>
+      <c r="G16" s="32"/>
+      <c r="H16" s="40"/>
+      <c r="I16" s="40"/>
+      <c r="J16" s="40"/>
       <c r="K16" s="9" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="17" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A17" s="28">
+      <c r="A17" s="37">
         <v>4</v>
       </c>
-      <c r="B17" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="C17" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="D17" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="E17" s="14" t="s">
+      <c r="B17" s="32" t="s">
+        <v>53</v>
+      </c>
+      <c r="C17" s="34" t="s">
+        <v>54</v>
+      </c>
+      <c r="D17" s="34" t="s">
+        <v>54</v>
+      </c>
+      <c r="E17" s="34" t="s">
         <v>54</v>
       </c>
       <c r="F17" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="G17" s="13" t="s">
-        <v>54</v>
-      </c>
-      <c r="H17" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="I17" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="J17" s="14" t="s">
+      <c r="G17" s="32" t="s">
+        <v>54</v>
+      </c>
+      <c r="H17" s="34" t="s">
+        <v>54</v>
+      </c>
+      <c r="I17" s="34" t="s">
+        <v>54</v>
+      </c>
+      <c r="J17" s="34" t="s">
         <v>54</v>
       </c>
       <c r="K17" s="9" t="s">
@@ -2929,85 +2932,85 @@
       </c>
     </row>
     <row r="18" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A18" s="29"/>
-      <c r="B18" s="13"/>
-      <c r="C18" s="17"/>
-      <c r="D18" s="17"/>
-      <c r="E18" s="17"/>
+      <c r="A18" s="38"/>
+      <c r="B18" s="32"/>
+      <c r="C18" s="40"/>
+      <c r="D18" s="40"/>
+      <c r="E18" s="40"/>
       <c r="F18" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="G18" s="13"/>
-      <c r="H18" s="17"/>
-      <c r="I18" s="17"/>
-      <c r="J18" s="17"/>
+      <c r="G18" s="32"/>
+      <c r="H18" s="40"/>
+      <c r="I18" s="40"/>
+      <c r="J18" s="40"/>
       <c r="K18" s="9" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="19" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A19" s="29"/>
-      <c r="B19" s="13"/>
-      <c r="C19" s="17"/>
-      <c r="D19" s="17"/>
-      <c r="E19" s="17"/>
+      <c r="A19" s="38"/>
+      <c r="B19" s="32"/>
+      <c r="C19" s="40"/>
+      <c r="D19" s="40"/>
+      <c r="E19" s="40"/>
       <c r="F19" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="G19" s="13"/>
-      <c r="H19" s="17"/>
-      <c r="I19" s="17"/>
-      <c r="J19" s="17"/>
+      <c r="G19" s="32"/>
+      <c r="H19" s="40"/>
+      <c r="I19" s="40"/>
+      <c r="J19" s="40"/>
       <c r="K19" s="9" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="20" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A20" s="30"/>
-      <c r="B20" s="13"/>
-      <c r="C20" s="17"/>
-      <c r="D20" s="17"/>
-      <c r="E20" s="17"/>
+      <c r="A20" s="39"/>
+      <c r="B20" s="32"/>
+      <c r="C20" s="40"/>
+      <c r="D20" s="40"/>
+      <c r="E20" s="40"/>
       <c r="F20" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="G20" s="13"/>
-      <c r="H20" s="17"/>
-      <c r="I20" s="17"/>
-      <c r="J20" s="17"/>
+      <c r="G20" s="32"/>
+      <c r="H20" s="40"/>
+      <c r="I20" s="40"/>
+      <c r="J20" s="40"/>
       <c r="K20" s="9" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="21" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A21" s="31">
+      <c r="A21" s="36">
         <v>5</v>
       </c>
-      <c r="B21" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="C21" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="D21" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="E21" s="14" t="s">
+      <c r="B21" s="32" t="s">
+        <v>53</v>
+      </c>
+      <c r="C21" s="34" t="s">
+        <v>53</v>
+      </c>
+      <c r="D21" s="34" t="s">
+        <v>54</v>
+      </c>
+      <c r="E21" s="34" t="s">
         <v>53</v>
       </c>
       <c r="F21" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="G21" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="H21" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="I21" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="J21" s="14" t="s">
+      <c r="G21" s="32" t="s">
+        <v>53</v>
+      </c>
+      <c r="H21" s="34" t="s">
+        <v>53</v>
+      </c>
+      <c r="I21" s="34" t="s">
+        <v>53</v>
+      </c>
+      <c r="J21" s="34" t="s">
         <v>53</v>
       </c>
       <c r="K21" s="9" t="s">
@@ -3015,85 +3018,85 @@
       </c>
     </row>
     <row r="22" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A22" s="32"/>
-      <c r="B22" s="13"/>
-      <c r="C22" s="14"/>
-      <c r="D22" s="14"/>
-      <c r="E22" s="14"/>
+      <c r="A22" s="30"/>
+      <c r="B22" s="32"/>
+      <c r="C22" s="34"/>
+      <c r="D22" s="34"/>
+      <c r="E22" s="34"/>
       <c r="F22" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="G22" s="13"/>
-      <c r="H22" s="14"/>
-      <c r="I22" s="14"/>
-      <c r="J22" s="14"/>
+      <c r="G22" s="32"/>
+      <c r="H22" s="34"/>
+      <c r="I22" s="34"/>
+      <c r="J22" s="34"/>
       <c r="K22" s="9" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="23" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A23" s="32"/>
-      <c r="B23" s="13"/>
-      <c r="C23" s="14"/>
-      <c r="D23" s="14"/>
-      <c r="E23" s="14"/>
+      <c r="A23" s="30"/>
+      <c r="B23" s="32"/>
+      <c r="C23" s="34"/>
+      <c r="D23" s="34"/>
+      <c r="E23" s="34"/>
       <c r="F23" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="G23" s="13"/>
-      <c r="H23" s="14"/>
-      <c r="I23" s="14"/>
-      <c r="J23" s="14"/>
+      <c r="G23" s="32"/>
+      <c r="H23" s="34"/>
+      <c r="I23" s="34"/>
+      <c r="J23" s="34"/>
       <c r="K23" s="9" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="24" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A24" s="33"/>
-      <c r="B24" s="13"/>
-      <c r="C24" s="14"/>
-      <c r="D24" s="14"/>
-      <c r="E24" s="14"/>
+      <c r="A24" s="41"/>
+      <c r="B24" s="32"/>
+      <c r="C24" s="34"/>
+      <c r="D24" s="34"/>
+      <c r="E24" s="34"/>
       <c r="F24" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="G24" s="13"/>
-      <c r="H24" s="14"/>
-      <c r="I24" s="14"/>
-      <c r="J24" s="14"/>
+      <c r="G24" s="32"/>
+      <c r="H24" s="34"/>
+      <c r="I24" s="34"/>
+      <c r="J24" s="34"/>
       <c r="K24" s="9" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="25" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A25" s="31">
+      <c r="A25" s="36">
         <v>6</v>
       </c>
-      <c r="B25" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="C25" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="D25" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="E25" s="14" t="s">
+      <c r="B25" s="32" t="s">
+        <v>53</v>
+      </c>
+      <c r="C25" s="34" t="s">
+        <v>54</v>
+      </c>
+      <c r="D25" s="34" t="s">
+        <v>53</v>
+      </c>
+      <c r="E25" s="34" t="s">
         <v>54</v>
       </c>
       <c r="F25" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="G25" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="H25" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="I25" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="J25" s="14" t="s">
+      <c r="G25" s="32" t="s">
+        <v>53</v>
+      </c>
+      <c r="H25" s="34" t="s">
+        <v>54</v>
+      </c>
+      <c r="I25" s="34" t="s">
+        <v>53</v>
+      </c>
+      <c r="J25" s="34" t="s">
         <v>54</v>
       </c>
       <c r="K25" s="9" t="s">
@@ -3101,85 +3104,85 @@
       </c>
     </row>
     <row r="26" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A26" s="32"/>
-      <c r="B26" s="13"/>
-      <c r="C26" s="14"/>
-      <c r="D26" s="14"/>
-      <c r="E26" s="14"/>
+      <c r="A26" s="30"/>
+      <c r="B26" s="32"/>
+      <c r="C26" s="34"/>
+      <c r="D26" s="34"/>
+      <c r="E26" s="34"/>
       <c r="F26" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="G26" s="13"/>
-      <c r="H26" s="14"/>
-      <c r="I26" s="14"/>
-      <c r="J26" s="14"/>
+      <c r="G26" s="32"/>
+      <c r="H26" s="34"/>
+      <c r="I26" s="34"/>
+      <c r="J26" s="34"/>
       <c r="K26" s="9" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="27" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A27" s="32"/>
-      <c r="B27" s="13"/>
-      <c r="C27" s="14"/>
-      <c r="D27" s="14"/>
-      <c r="E27" s="14"/>
+      <c r="A27" s="30"/>
+      <c r="B27" s="32"/>
+      <c r="C27" s="34"/>
+      <c r="D27" s="34"/>
+      <c r="E27" s="34"/>
       <c r="F27" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="G27" s="13"/>
-      <c r="H27" s="14"/>
-      <c r="I27" s="14"/>
-      <c r="J27" s="14"/>
+      <c r="G27" s="32"/>
+      <c r="H27" s="34"/>
+      <c r="I27" s="34"/>
+      <c r="J27" s="34"/>
       <c r="K27" s="9" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="28" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A28" s="35"/>
-      <c r="B28" s="13"/>
-      <c r="C28" s="14"/>
-      <c r="D28" s="14"/>
-      <c r="E28" s="14"/>
+      <c r="A28" s="31"/>
+      <c r="B28" s="32"/>
+      <c r="C28" s="34"/>
+      <c r="D28" s="34"/>
+      <c r="E28" s="34"/>
       <c r="F28" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="G28" s="13"/>
-      <c r="H28" s="14"/>
-      <c r="I28" s="14"/>
-      <c r="J28" s="14"/>
+      <c r="G28" s="32"/>
+      <c r="H28" s="34"/>
+      <c r="I28" s="34"/>
+      <c r="J28" s="34"/>
       <c r="K28" s="9" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="29" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A29" s="34">
+      <c r="A29" s="29">
         <v>7</v>
       </c>
-      <c r="B29" s="13" t="s">
-        <v>54</v>
-      </c>
-      <c r="C29" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="D29" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="E29" s="14" t="s">
+      <c r="B29" s="32" t="s">
+        <v>54</v>
+      </c>
+      <c r="C29" s="34" t="s">
+        <v>53</v>
+      </c>
+      <c r="D29" s="34" t="s">
+        <v>54</v>
+      </c>
+      <c r="E29" s="34" t="s">
         <v>54</v>
       </c>
       <c r="F29" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="G29" s="13" t="s">
-        <v>54</v>
-      </c>
-      <c r="H29" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="I29" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="J29" s="14" t="s">
+      <c r="G29" s="32" t="s">
+        <v>54</v>
+      </c>
+      <c r="H29" s="34" t="s">
+        <v>54</v>
+      </c>
+      <c r="I29" s="34" t="s">
+        <v>53</v>
+      </c>
+      <c r="J29" s="34" t="s">
         <v>53</v>
       </c>
       <c r="K29" s="9" t="s">
@@ -3187,85 +3190,85 @@
       </c>
     </row>
     <row r="30" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A30" s="32"/>
-      <c r="B30" s="13"/>
-      <c r="C30" s="14"/>
-      <c r="D30" s="14"/>
-      <c r="E30" s="14"/>
+      <c r="A30" s="30"/>
+      <c r="B30" s="32"/>
+      <c r="C30" s="34"/>
+      <c r="D30" s="34"/>
+      <c r="E30" s="34"/>
       <c r="F30" s="12" t="s">
         <v>82</v>
       </c>
-      <c r="G30" s="13"/>
-      <c r="H30" s="14"/>
-      <c r="I30" s="14"/>
-      <c r="J30" s="14"/>
+      <c r="G30" s="32"/>
+      <c r="H30" s="34"/>
+      <c r="I30" s="34"/>
+      <c r="J30" s="34"/>
       <c r="K30" s="9" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="31" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A31" s="32"/>
-      <c r="B31" s="13"/>
-      <c r="C31" s="14"/>
-      <c r="D31" s="14"/>
-      <c r="E31" s="14"/>
+      <c r="A31" s="30"/>
+      <c r="B31" s="32"/>
+      <c r="C31" s="34"/>
+      <c r="D31" s="34"/>
+      <c r="E31" s="34"/>
       <c r="F31" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="G31" s="13"/>
-      <c r="H31" s="14"/>
-      <c r="I31" s="14"/>
-      <c r="J31" s="14"/>
+      <c r="G31" s="32"/>
+      <c r="H31" s="34"/>
+      <c r="I31" s="34"/>
+      <c r="J31" s="34"/>
       <c r="K31" s="9" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="32" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A32" s="35"/>
-      <c r="B32" s="13"/>
-      <c r="C32" s="14"/>
-      <c r="D32" s="14"/>
-      <c r="E32" s="14"/>
+      <c r="A32" s="31"/>
+      <c r="B32" s="32"/>
+      <c r="C32" s="34"/>
+      <c r="D32" s="34"/>
+      <c r="E32" s="34"/>
       <c r="F32" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="G32" s="13"/>
-      <c r="H32" s="14"/>
-      <c r="I32" s="14"/>
-      <c r="J32" s="14"/>
+      <c r="G32" s="32"/>
+      <c r="H32" s="34"/>
+      <c r="I32" s="34"/>
+      <c r="J32" s="34"/>
       <c r="K32" s="9" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="33" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A33" s="34">
+      <c r="A33" s="29">
         <v>8</v>
       </c>
-      <c r="B33" s="13" t="s">
-        <v>54</v>
-      </c>
-      <c r="C33" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="D33" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="E33" s="14" t="s">
+      <c r="B33" s="32" t="s">
+        <v>54</v>
+      </c>
+      <c r="C33" s="34" t="s">
+        <v>53</v>
+      </c>
+      <c r="D33" s="34" t="s">
+        <v>54</v>
+      </c>
+      <c r="E33" s="34" t="s">
         <v>54</v>
       </c>
       <c r="F33" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="G33" s="13" t="s">
-        <v>54</v>
-      </c>
-      <c r="H33" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="I33" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="J33" s="14" t="s">
+      <c r="G33" s="32" t="s">
+        <v>54</v>
+      </c>
+      <c r="H33" s="34" t="s">
+        <v>54</v>
+      </c>
+      <c r="I33" s="34" t="s">
+        <v>54</v>
+      </c>
+      <c r="J33" s="34" t="s">
         <v>54</v>
       </c>
       <c r="K33" s="9" t="s">
@@ -3273,85 +3276,85 @@
       </c>
     </row>
     <row r="34" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A34" s="32"/>
-      <c r="B34" s="13"/>
-      <c r="C34" s="14"/>
-      <c r="D34" s="14"/>
-      <c r="E34" s="14"/>
+      <c r="A34" s="30"/>
+      <c r="B34" s="32"/>
+      <c r="C34" s="34"/>
+      <c r="D34" s="34"/>
+      <c r="E34" s="34"/>
       <c r="F34" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="G34" s="13"/>
-      <c r="H34" s="14"/>
-      <c r="I34" s="14"/>
-      <c r="J34" s="14"/>
+      <c r="G34" s="32"/>
+      <c r="H34" s="34"/>
+      <c r="I34" s="34"/>
+      <c r="J34" s="34"/>
       <c r="K34" s="9" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="35" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A35" s="32"/>
-      <c r="B35" s="13"/>
-      <c r="C35" s="14"/>
-      <c r="D35" s="14"/>
-      <c r="E35" s="14"/>
+      <c r="A35" s="30"/>
+      <c r="B35" s="32"/>
+      <c r="C35" s="34"/>
+      <c r="D35" s="34"/>
+      <c r="E35" s="34"/>
       <c r="F35" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="G35" s="13"/>
-      <c r="H35" s="14"/>
-      <c r="I35" s="14"/>
-      <c r="J35" s="14"/>
+      <c r="G35" s="32"/>
+      <c r="H35" s="34"/>
+      <c r="I35" s="34"/>
+      <c r="J35" s="34"/>
       <c r="K35" s="9" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="36" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A36" s="35"/>
-      <c r="B36" s="13"/>
-      <c r="C36" s="14"/>
-      <c r="D36" s="14"/>
-      <c r="E36" s="14"/>
+      <c r="A36" s="31"/>
+      <c r="B36" s="32"/>
+      <c r="C36" s="34"/>
+      <c r="D36" s="34"/>
+      <c r="E36" s="34"/>
       <c r="F36" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="G36" s="13"/>
-      <c r="H36" s="14"/>
-      <c r="I36" s="14"/>
-      <c r="J36" s="14"/>
+      <c r="G36" s="32"/>
+      <c r="H36" s="34"/>
+      <c r="I36" s="34"/>
+      <c r="J36" s="34"/>
       <c r="K36" s="9" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="37" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A37" s="34">
+      <c r="A37" s="29">
         <v>9</v>
       </c>
-      <c r="B37" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="C37" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="D37" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="E37" s="14" t="s">
+      <c r="B37" s="32" t="s">
+        <v>53</v>
+      </c>
+      <c r="C37" s="34" t="s">
+        <v>53</v>
+      </c>
+      <c r="D37" s="34" t="s">
+        <v>54</v>
+      </c>
+      <c r="E37" s="34" t="s">
         <v>54</v>
       </c>
       <c r="F37" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="G37" s="13" t="s">
-        <v>54</v>
-      </c>
-      <c r="H37" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="I37" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="J37" s="14" t="s">
+      <c r="G37" s="32" t="s">
+        <v>54</v>
+      </c>
+      <c r="H37" s="34" t="s">
+        <v>54</v>
+      </c>
+      <c r="I37" s="34" t="s">
+        <v>54</v>
+      </c>
+      <c r="J37" s="34" t="s">
         <v>54</v>
       </c>
       <c r="K37" s="9" t="s">
@@ -3359,85 +3362,85 @@
       </c>
     </row>
     <row r="38" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A38" s="32"/>
-      <c r="B38" s="13"/>
-      <c r="C38" s="14"/>
-      <c r="D38" s="14"/>
-      <c r="E38" s="14"/>
+      <c r="A38" s="30"/>
+      <c r="B38" s="32"/>
+      <c r="C38" s="34"/>
+      <c r="D38" s="34"/>
+      <c r="E38" s="34"/>
       <c r="F38" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="G38" s="13"/>
-      <c r="H38" s="14"/>
-      <c r="I38" s="14"/>
-      <c r="J38" s="14"/>
+      <c r="G38" s="32"/>
+      <c r="H38" s="34"/>
+      <c r="I38" s="34"/>
+      <c r="J38" s="34"/>
       <c r="K38" s="9" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="39" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A39" s="32"/>
-      <c r="B39" s="13"/>
-      <c r="C39" s="14"/>
-      <c r="D39" s="14"/>
-      <c r="E39" s="14"/>
+      <c r="A39" s="30"/>
+      <c r="B39" s="32"/>
+      <c r="C39" s="34"/>
+      <c r="D39" s="34"/>
+      <c r="E39" s="34"/>
       <c r="F39" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="G39" s="13"/>
-      <c r="H39" s="14"/>
-      <c r="I39" s="14"/>
-      <c r="J39" s="14"/>
+      <c r="G39" s="32"/>
+      <c r="H39" s="34"/>
+      <c r="I39" s="34"/>
+      <c r="J39" s="34"/>
       <c r="K39" s="9" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="40" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A40" s="35"/>
-      <c r="B40" s="13"/>
-      <c r="C40" s="14"/>
-      <c r="D40" s="14"/>
-      <c r="E40" s="14"/>
+      <c r="A40" s="31"/>
+      <c r="B40" s="32"/>
+      <c r="C40" s="34"/>
+      <c r="D40" s="34"/>
+      <c r="E40" s="34"/>
       <c r="F40" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="G40" s="13"/>
-      <c r="H40" s="14"/>
-      <c r="I40" s="14"/>
-      <c r="J40" s="14"/>
+      <c r="G40" s="32"/>
+      <c r="H40" s="34"/>
+      <c r="I40" s="34"/>
+      <c r="J40" s="34"/>
       <c r="K40" s="9" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="41" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A41" s="34">
+      <c r="A41" s="29">
         <v>10</v>
       </c>
-      <c r="B41" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="C41" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="D41" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="E41" s="14" t="s">
+      <c r="B41" s="32" t="s">
+        <v>53</v>
+      </c>
+      <c r="C41" s="34" t="s">
+        <v>54</v>
+      </c>
+      <c r="D41" s="34" t="s">
+        <v>53</v>
+      </c>
+      <c r="E41" s="34" t="s">
         <v>53</v>
       </c>
       <c r="F41" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="G41" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="H41" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="I41" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="J41" s="14" t="s">
+      <c r="G41" s="32" t="s">
+        <v>53</v>
+      </c>
+      <c r="H41" s="34" t="s">
+        <v>53</v>
+      </c>
+      <c r="I41" s="34" t="s">
+        <v>53</v>
+      </c>
+      <c r="J41" s="34" t="s">
         <v>53</v>
       </c>
       <c r="K41" s="9" t="s">
@@ -3445,85 +3448,85 @@
       </c>
     </row>
     <row r="42" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A42" s="32"/>
-      <c r="B42" s="13"/>
-      <c r="C42" s="14"/>
-      <c r="D42" s="14"/>
-      <c r="E42" s="14"/>
+      <c r="A42" s="30"/>
+      <c r="B42" s="32"/>
+      <c r="C42" s="34"/>
+      <c r="D42" s="34"/>
+      <c r="E42" s="34"/>
       <c r="F42" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="G42" s="13"/>
-      <c r="H42" s="14"/>
-      <c r="I42" s="14"/>
-      <c r="J42" s="14"/>
+      <c r="G42" s="32"/>
+      <c r="H42" s="34"/>
+      <c r="I42" s="34"/>
+      <c r="J42" s="34"/>
       <c r="K42" s="9" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="43" spans="1:11" ht="28" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A43" s="32"/>
-      <c r="B43" s="13"/>
-      <c r="C43" s="14"/>
-      <c r="D43" s="14"/>
-      <c r="E43" s="14"/>
+      <c r="A43" s="30"/>
+      <c r="B43" s="32"/>
+      <c r="C43" s="34"/>
+      <c r="D43" s="34"/>
+      <c r="E43" s="34"/>
       <c r="F43" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="G43" s="13"/>
-      <c r="H43" s="14"/>
-      <c r="I43" s="14"/>
-      <c r="J43" s="14"/>
+      <c r="G43" s="32"/>
+      <c r="H43" s="34"/>
+      <c r="I43" s="34"/>
+      <c r="J43" s="34"/>
       <c r="K43" s="9" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="44" spans="1:11" ht="28" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A44" s="35"/>
-      <c r="B44" s="13"/>
-      <c r="C44" s="14"/>
-      <c r="D44" s="14"/>
-      <c r="E44" s="14"/>
+      <c r="A44" s="31"/>
+      <c r="B44" s="32"/>
+      <c r="C44" s="34"/>
+      <c r="D44" s="34"/>
+      <c r="E44" s="34"/>
       <c r="F44" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="G44" s="13"/>
-      <c r="H44" s="14"/>
-      <c r="I44" s="14"/>
-      <c r="J44" s="14"/>
+      <c r="G44" s="32"/>
+      <c r="H44" s="34"/>
+      <c r="I44" s="34"/>
+      <c r="J44" s="34"/>
       <c r="K44" s="9" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="45" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A45" s="34">
+      <c r="A45" s="29">
         <v>11</v>
       </c>
-      <c r="B45" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="C45" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="D45" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="E45" s="14" t="s">
+      <c r="B45" s="32" t="s">
+        <v>53</v>
+      </c>
+      <c r="C45" s="34" t="s">
+        <v>53</v>
+      </c>
+      <c r="D45" s="34" t="s">
+        <v>53</v>
+      </c>
+      <c r="E45" s="34" t="s">
         <v>53</v>
       </c>
       <c r="F45" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="G45" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="H45" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="I45" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="J45" s="14" t="s">
+      <c r="G45" s="32" t="s">
+        <v>53</v>
+      </c>
+      <c r="H45" s="34" t="s">
+        <v>53</v>
+      </c>
+      <c r="I45" s="34" t="s">
+        <v>53</v>
+      </c>
+      <c r="J45" s="34" t="s">
         <v>53</v>
       </c>
       <c r="K45" s="9" t="s">
@@ -3531,85 +3534,85 @@
       </c>
     </row>
     <row r="46" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A46" s="32"/>
-      <c r="B46" s="13"/>
-      <c r="C46" s="14"/>
-      <c r="D46" s="14"/>
-      <c r="E46" s="14"/>
+      <c r="A46" s="30"/>
+      <c r="B46" s="32"/>
+      <c r="C46" s="34"/>
+      <c r="D46" s="34"/>
+      <c r="E46" s="34"/>
       <c r="F46" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="G46" s="13"/>
-      <c r="H46" s="14"/>
-      <c r="I46" s="14"/>
-      <c r="J46" s="14"/>
+      <c r="G46" s="32"/>
+      <c r="H46" s="34"/>
+      <c r="I46" s="34"/>
+      <c r="J46" s="34"/>
       <c r="K46" s="9" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="47" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A47" s="32"/>
-      <c r="B47" s="13"/>
-      <c r="C47" s="14"/>
-      <c r="D47" s="14"/>
-      <c r="E47" s="14"/>
+      <c r="A47" s="30"/>
+      <c r="B47" s="32"/>
+      <c r="C47" s="34"/>
+      <c r="D47" s="34"/>
+      <c r="E47" s="34"/>
       <c r="F47" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="G47" s="13"/>
-      <c r="H47" s="14"/>
-      <c r="I47" s="14"/>
-      <c r="J47" s="14"/>
+      <c r="G47" s="32"/>
+      <c r="H47" s="34"/>
+      <c r="I47" s="34"/>
+      <c r="J47" s="34"/>
       <c r="K47" s="9" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="48" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A48" s="35"/>
-      <c r="B48" s="13"/>
-      <c r="C48" s="14"/>
-      <c r="D48" s="14"/>
-      <c r="E48" s="14"/>
+      <c r="A48" s="31"/>
+      <c r="B48" s="32"/>
+      <c r="C48" s="34"/>
+      <c r="D48" s="34"/>
+      <c r="E48" s="34"/>
       <c r="F48" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="G48" s="13"/>
-      <c r="H48" s="14"/>
-      <c r="I48" s="14"/>
-      <c r="J48" s="14"/>
+      <c r="G48" s="32"/>
+      <c r="H48" s="34"/>
+      <c r="I48" s="34"/>
+      <c r="J48" s="34"/>
       <c r="K48" s="9" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="49" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A49" s="34">
+      <c r="A49" s="29">
         <v>12</v>
       </c>
-      <c r="B49" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="C49" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="D49" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="E49" s="14" t="s">
+      <c r="B49" s="32" t="s">
+        <v>53</v>
+      </c>
+      <c r="C49" s="34" t="s">
+        <v>53</v>
+      </c>
+      <c r="D49" s="34" t="s">
+        <v>53</v>
+      </c>
+      <c r="E49" s="34" t="s">
         <v>53</v>
       </c>
       <c r="F49" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="G49" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="H49" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="I49" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="J49" s="14" t="s">
+      <c r="G49" s="32" t="s">
+        <v>53</v>
+      </c>
+      <c r="H49" s="34" t="s">
+        <v>53</v>
+      </c>
+      <c r="I49" s="34" t="s">
+        <v>53</v>
+      </c>
+      <c r="J49" s="34" t="s">
         <v>53</v>
       </c>
       <c r="K49" s="9" t="s">
@@ -3617,85 +3620,85 @@
       </c>
     </row>
     <row r="50" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A50" s="32"/>
-      <c r="B50" s="13"/>
-      <c r="C50" s="14"/>
-      <c r="D50" s="14"/>
-      <c r="E50" s="14"/>
+      <c r="A50" s="30"/>
+      <c r="B50" s="32"/>
+      <c r="C50" s="34"/>
+      <c r="D50" s="34"/>
+      <c r="E50" s="34"/>
       <c r="F50" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="G50" s="13"/>
-      <c r="H50" s="14"/>
-      <c r="I50" s="14"/>
-      <c r="J50" s="14"/>
+      <c r="G50" s="32"/>
+      <c r="H50" s="34"/>
+      <c r="I50" s="34"/>
+      <c r="J50" s="34"/>
       <c r="K50" s="9" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="51" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A51" s="32"/>
-      <c r="B51" s="13"/>
-      <c r="C51" s="14"/>
-      <c r="D51" s="14"/>
-      <c r="E51" s="14"/>
+      <c r="A51" s="30"/>
+      <c r="B51" s="32"/>
+      <c r="C51" s="34"/>
+      <c r="D51" s="34"/>
+      <c r="E51" s="34"/>
       <c r="F51" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="G51" s="13"/>
-      <c r="H51" s="14"/>
-      <c r="I51" s="14"/>
-      <c r="J51" s="14"/>
+      <c r="G51" s="32"/>
+      <c r="H51" s="34"/>
+      <c r="I51" s="34"/>
+      <c r="J51" s="34"/>
       <c r="K51" s="9" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="52" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A52" s="35"/>
-      <c r="B52" s="13"/>
-      <c r="C52" s="14"/>
-      <c r="D52" s="14"/>
-      <c r="E52" s="14"/>
+      <c r="A52" s="31"/>
+      <c r="B52" s="32"/>
+      <c r="C52" s="34"/>
+      <c r="D52" s="34"/>
+      <c r="E52" s="34"/>
       <c r="F52" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="G52" s="13"/>
-      <c r="H52" s="14"/>
-      <c r="I52" s="14"/>
-      <c r="J52" s="14"/>
+      <c r="G52" s="32"/>
+      <c r="H52" s="34"/>
+      <c r="I52" s="34"/>
+      <c r="J52" s="34"/>
       <c r="K52" s="9" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="53" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A53" s="34">
+      <c r="A53" s="29">
         <v>13</v>
       </c>
-      <c r="B53" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="C53" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="D53" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="E53" s="14" t="s">
+      <c r="B53" s="32" t="s">
+        <v>53</v>
+      </c>
+      <c r="C53" s="34" t="s">
+        <v>54</v>
+      </c>
+      <c r="D53" s="34" t="s">
+        <v>54</v>
+      </c>
+      <c r="E53" s="34" t="s">
         <v>54</v>
       </c>
       <c r="F53" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="G53" s="13" t="s">
-        <v>54</v>
-      </c>
-      <c r="H53" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="I53" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="J53" s="14" t="s">
+      <c r="G53" s="32" t="s">
+        <v>54</v>
+      </c>
+      <c r="H53" s="34" t="s">
+        <v>54</v>
+      </c>
+      <c r="I53" s="34" t="s">
+        <v>54</v>
+      </c>
+      <c r="J53" s="34" t="s">
         <v>54</v>
       </c>
       <c r="K53" s="9" t="s">
@@ -3703,85 +3706,85 @@
       </c>
     </row>
     <row r="54" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A54" s="32"/>
-      <c r="B54" s="13"/>
-      <c r="C54" s="14"/>
-      <c r="D54" s="14"/>
-      <c r="E54" s="14"/>
+      <c r="A54" s="30"/>
+      <c r="B54" s="32"/>
+      <c r="C54" s="34"/>
+      <c r="D54" s="34"/>
+      <c r="E54" s="34"/>
       <c r="F54" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="G54" s="13"/>
-      <c r="H54" s="14"/>
-      <c r="I54" s="14"/>
-      <c r="J54" s="14"/>
+      <c r="G54" s="32"/>
+      <c r="H54" s="34"/>
+      <c r="I54" s="34"/>
+      <c r="J54" s="34"/>
       <c r="K54" s="9" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="55" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A55" s="32"/>
-      <c r="B55" s="13"/>
-      <c r="C55" s="14"/>
-      <c r="D55" s="14"/>
-      <c r="E55" s="14"/>
+      <c r="A55" s="30"/>
+      <c r="B55" s="32"/>
+      <c r="C55" s="34"/>
+      <c r="D55" s="34"/>
+      <c r="E55" s="34"/>
       <c r="F55" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="G55" s="13"/>
-      <c r="H55" s="14"/>
-      <c r="I55" s="14"/>
-      <c r="J55" s="14"/>
+      <c r="G55" s="32"/>
+      <c r="H55" s="34"/>
+      <c r="I55" s="34"/>
+      <c r="J55" s="34"/>
       <c r="K55" s="9" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="56" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A56" s="35"/>
-      <c r="B56" s="13"/>
-      <c r="C56" s="14"/>
-      <c r="D56" s="14"/>
-      <c r="E56" s="14"/>
+      <c r="A56" s="31"/>
+      <c r="B56" s="32"/>
+      <c r="C56" s="34"/>
+      <c r="D56" s="34"/>
+      <c r="E56" s="34"/>
       <c r="F56" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="G56" s="13"/>
-      <c r="H56" s="14"/>
-      <c r="I56" s="14"/>
-      <c r="J56" s="14"/>
+      <c r="G56" s="32"/>
+      <c r="H56" s="34"/>
+      <c r="I56" s="34"/>
+      <c r="J56" s="34"/>
       <c r="K56" s="9" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="57" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A57" s="34">
+      <c r="A57" s="29">
         <v>14</v>
       </c>
-      <c r="B57" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="C57" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="D57" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="E57" s="14" t="s">
+      <c r="B57" s="32" t="s">
+        <v>53</v>
+      </c>
+      <c r="C57" s="34" t="s">
+        <v>54</v>
+      </c>
+      <c r="D57" s="34" t="s">
+        <v>54</v>
+      </c>
+      <c r="E57" s="34" t="s">
         <v>53</v>
       </c>
       <c r="F57" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="G57" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="H57" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="I57" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="J57" s="14" t="s">
+      <c r="G57" s="32" t="s">
+        <v>53</v>
+      </c>
+      <c r="H57" s="34" t="s">
+        <v>54</v>
+      </c>
+      <c r="I57" s="34" t="s">
+        <v>53</v>
+      </c>
+      <c r="J57" s="34" t="s">
         <v>53</v>
       </c>
       <c r="K57" s="9" t="s">
@@ -3789,85 +3792,85 @@
       </c>
     </row>
     <row r="58" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A58" s="32"/>
-      <c r="B58" s="13"/>
-      <c r="C58" s="14"/>
-      <c r="D58" s="14"/>
-      <c r="E58" s="14"/>
+      <c r="A58" s="30"/>
+      <c r="B58" s="32"/>
+      <c r="C58" s="34"/>
+      <c r="D58" s="34"/>
+      <c r="E58" s="34"/>
       <c r="F58" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="G58" s="13"/>
-      <c r="H58" s="14"/>
-      <c r="I58" s="14"/>
-      <c r="J58" s="14"/>
+      <c r="G58" s="32"/>
+      <c r="H58" s="34"/>
+      <c r="I58" s="34"/>
+      <c r="J58" s="34"/>
       <c r="K58" s="9" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="59" spans="1:11" ht="42" x14ac:dyDescent="0.15">
-      <c r="A59" s="32"/>
-      <c r="B59" s="13"/>
-      <c r="C59" s="14"/>
-      <c r="D59" s="14"/>
-      <c r="E59" s="14"/>
+      <c r="A59" s="30"/>
+      <c r="B59" s="32"/>
+      <c r="C59" s="34"/>
+      <c r="D59" s="34"/>
+      <c r="E59" s="34"/>
       <c r="F59" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="G59" s="13"/>
-      <c r="H59" s="14"/>
-      <c r="I59" s="14"/>
-      <c r="J59" s="14"/>
+      <c r="G59" s="32"/>
+      <c r="H59" s="34"/>
+      <c r="I59" s="34"/>
+      <c r="J59" s="34"/>
       <c r="K59" s="9" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="60" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A60" s="35"/>
-      <c r="B60" s="13"/>
-      <c r="C60" s="14"/>
-      <c r="D60" s="14"/>
-      <c r="E60" s="14"/>
+      <c r="A60" s="31"/>
+      <c r="B60" s="32"/>
+      <c r="C60" s="34"/>
+      <c r="D60" s="34"/>
+      <c r="E60" s="34"/>
       <c r="F60" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="G60" s="13"/>
-      <c r="H60" s="14"/>
-      <c r="I60" s="14"/>
-      <c r="J60" s="14"/>
+      <c r="G60" s="32"/>
+      <c r="H60" s="34"/>
+      <c r="I60" s="34"/>
+      <c r="J60" s="34"/>
       <c r="K60" s="9" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="61" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A61" s="34">
+      <c r="A61" s="29">
         <v>15</v>
       </c>
-      <c r="B61" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="C61" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="D61" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="E61" s="14" t="s">
+      <c r="B61" s="32" t="s">
+        <v>53</v>
+      </c>
+      <c r="C61" s="34" t="s">
+        <v>54</v>
+      </c>
+      <c r="D61" s="34" t="s">
+        <v>54</v>
+      </c>
+      <c r="E61" s="34" t="s">
         <v>54</v>
       </c>
       <c r="F61" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="G61" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="H61" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="I61" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="J61" s="14" t="s">
+      <c r="G61" s="32" t="s">
+        <v>53</v>
+      </c>
+      <c r="H61" s="34" t="s">
+        <v>53</v>
+      </c>
+      <c r="I61" s="34" t="s">
+        <v>53</v>
+      </c>
+      <c r="J61" s="34" t="s">
         <v>53</v>
       </c>
       <c r="K61" s="9" t="s">
@@ -3875,108 +3878,128 @@
       </c>
     </row>
     <row r="62" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A62" s="32"/>
-      <c r="B62" s="13"/>
-      <c r="C62" s="14"/>
-      <c r="D62" s="14"/>
-      <c r="E62" s="14"/>
+      <c r="A62" s="30"/>
+      <c r="B62" s="32"/>
+      <c r="C62" s="34"/>
+      <c r="D62" s="34"/>
+      <c r="E62" s="34"/>
       <c r="F62" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="G62" s="13"/>
-      <c r="H62" s="14"/>
-      <c r="I62" s="14"/>
-      <c r="J62" s="14"/>
+      <c r="G62" s="32"/>
+      <c r="H62" s="34"/>
+      <c r="I62" s="34"/>
+      <c r="J62" s="34"/>
       <c r="K62" s="9" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="63" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A63" s="32"/>
-      <c r="B63" s="13"/>
-      <c r="C63" s="14"/>
-      <c r="D63" s="14"/>
-      <c r="E63" s="14"/>
+      <c r="A63" s="30"/>
+      <c r="B63" s="32"/>
+      <c r="C63" s="34"/>
+      <c r="D63" s="34"/>
+      <c r="E63" s="34"/>
       <c r="F63" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="G63" s="13"/>
-      <c r="H63" s="14"/>
-      <c r="I63" s="14"/>
-      <c r="J63" s="14"/>
+      <c r="G63" s="32"/>
+      <c r="H63" s="34"/>
+      <c r="I63" s="34"/>
+      <c r="J63" s="34"/>
       <c r="K63" s="9" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="64" spans="1:11" ht="14" x14ac:dyDescent="0.15">
-      <c r="A64" s="35"/>
-      <c r="B64" s="15"/>
-      <c r="C64" s="16"/>
-      <c r="D64" s="16"/>
-      <c r="E64" s="16"/>
+      <c r="A64" s="31"/>
+      <c r="B64" s="33"/>
+      <c r="C64" s="35"/>
+      <c r="D64" s="35"/>
+      <c r="E64" s="35"/>
       <c r="F64" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="G64" s="15"/>
-      <c r="H64" s="16"/>
-      <c r="I64" s="16"/>
-      <c r="J64" s="16"/>
+      <c r="G64" s="33"/>
+      <c r="H64" s="35"/>
+      <c r="I64" s="35"/>
+      <c r="J64" s="35"/>
       <c r="K64" s="10" t="s">
         <v>57</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="144">
-    <mergeCell ref="A61:A64"/>
-    <mergeCell ref="B61:B64"/>
-    <mergeCell ref="C61:C64"/>
-    <mergeCell ref="D61:D64"/>
-    <mergeCell ref="E61:E64"/>
-    <mergeCell ref="A57:A60"/>
-    <mergeCell ref="B57:B60"/>
-    <mergeCell ref="C57:C60"/>
-    <mergeCell ref="D57:D60"/>
-    <mergeCell ref="E57:E60"/>
-    <mergeCell ref="A53:A56"/>
-    <mergeCell ref="B53:B56"/>
-    <mergeCell ref="C53:C56"/>
-    <mergeCell ref="D53:D56"/>
-    <mergeCell ref="E53:E56"/>
-    <mergeCell ref="A49:A52"/>
-    <mergeCell ref="B49:B52"/>
-    <mergeCell ref="C49:C52"/>
-    <mergeCell ref="D49:D52"/>
-    <mergeCell ref="E49:E52"/>
-    <mergeCell ref="A45:A48"/>
-    <mergeCell ref="B45:B48"/>
-    <mergeCell ref="C45:C48"/>
-    <mergeCell ref="D45:D48"/>
-    <mergeCell ref="E45:E48"/>
-    <mergeCell ref="A41:A44"/>
-    <mergeCell ref="B41:B44"/>
-    <mergeCell ref="C41:C44"/>
-    <mergeCell ref="E41:E44"/>
-    <mergeCell ref="D41:D44"/>
-    <mergeCell ref="A37:A40"/>
-    <mergeCell ref="B37:B40"/>
-    <mergeCell ref="C37:C40"/>
-    <mergeCell ref="D37:D40"/>
-    <mergeCell ref="E37:E40"/>
-    <mergeCell ref="A33:A36"/>
-    <mergeCell ref="B33:B36"/>
-    <mergeCell ref="C33:C36"/>
-    <mergeCell ref="D33:D36"/>
-    <mergeCell ref="E33:E36"/>
-    <mergeCell ref="A29:A32"/>
-    <mergeCell ref="B29:B32"/>
-    <mergeCell ref="C29:C32"/>
-    <mergeCell ref="D29:D32"/>
-    <mergeCell ref="E29:E32"/>
-    <mergeCell ref="A25:A28"/>
-    <mergeCell ref="B25:B28"/>
-    <mergeCell ref="C25:C28"/>
-    <mergeCell ref="D25:D28"/>
-    <mergeCell ref="E25:E28"/>
+    <mergeCell ref="G57:G60"/>
+    <mergeCell ref="H57:H60"/>
+    <mergeCell ref="I57:I60"/>
+    <mergeCell ref="J57:J60"/>
+    <mergeCell ref="G61:G64"/>
+    <mergeCell ref="H61:H64"/>
+    <mergeCell ref="I61:I64"/>
+    <mergeCell ref="J61:J64"/>
+    <mergeCell ref="G49:G52"/>
+    <mergeCell ref="H49:H52"/>
+    <mergeCell ref="I49:I52"/>
+    <mergeCell ref="J49:J52"/>
+    <mergeCell ref="G53:G56"/>
+    <mergeCell ref="H53:H56"/>
+    <mergeCell ref="I53:I56"/>
+    <mergeCell ref="J53:J56"/>
+    <mergeCell ref="G41:G44"/>
+    <mergeCell ref="H41:H44"/>
+    <mergeCell ref="I41:I44"/>
+    <mergeCell ref="J41:J44"/>
+    <mergeCell ref="G45:G48"/>
+    <mergeCell ref="H45:H48"/>
+    <mergeCell ref="I45:I48"/>
+    <mergeCell ref="J45:J48"/>
+    <mergeCell ref="G33:G36"/>
+    <mergeCell ref="H33:H36"/>
+    <mergeCell ref="I33:I36"/>
+    <mergeCell ref="J33:J36"/>
+    <mergeCell ref="G37:G40"/>
+    <mergeCell ref="H37:H40"/>
+    <mergeCell ref="I37:I40"/>
+    <mergeCell ref="J37:J40"/>
+    <mergeCell ref="G25:G28"/>
+    <mergeCell ref="H25:H28"/>
+    <mergeCell ref="I25:I28"/>
+    <mergeCell ref="J25:J28"/>
+    <mergeCell ref="G29:G32"/>
+    <mergeCell ref="H29:H32"/>
+    <mergeCell ref="I29:I32"/>
+    <mergeCell ref="J29:J32"/>
+    <mergeCell ref="G17:G20"/>
+    <mergeCell ref="H17:H20"/>
+    <mergeCell ref="I17:I20"/>
+    <mergeCell ref="J17:J20"/>
+    <mergeCell ref="G21:G24"/>
+    <mergeCell ref="H21:H24"/>
+    <mergeCell ref="I21:I24"/>
+    <mergeCell ref="J21:J24"/>
+    <mergeCell ref="G9:G12"/>
+    <mergeCell ref="H9:H12"/>
+    <mergeCell ref="I9:I12"/>
+    <mergeCell ref="J9:J12"/>
+    <mergeCell ref="G13:G16"/>
+    <mergeCell ref="H13:H16"/>
+    <mergeCell ref="I13:I16"/>
+    <mergeCell ref="J13:J16"/>
+    <mergeCell ref="B2:F2"/>
+    <mergeCell ref="G3:H3"/>
+    <mergeCell ref="I3:J3"/>
+    <mergeCell ref="E9:E12"/>
+    <mergeCell ref="K3:K4"/>
+    <mergeCell ref="G5:G8"/>
+    <mergeCell ref="H5:H8"/>
+    <mergeCell ref="I5:I8"/>
+    <mergeCell ref="J5:J8"/>
+    <mergeCell ref="G2:K2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="F3:F4"/>
     <mergeCell ref="A13:A16"/>
     <mergeCell ref="B13:B16"/>
     <mergeCell ref="C13:C16"/>
@@ -4001,76 +4024,56 @@
     <mergeCell ref="B9:B12"/>
     <mergeCell ref="C9:C12"/>
     <mergeCell ref="D9:D12"/>
-    <mergeCell ref="K3:K4"/>
-    <mergeCell ref="G5:G8"/>
-    <mergeCell ref="H5:H8"/>
-    <mergeCell ref="I5:I8"/>
-    <mergeCell ref="J5:J8"/>
-    <mergeCell ref="G2:K2"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="F3:F4"/>
-    <mergeCell ref="G9:G12"/>
-    <mergeCell ref="H9:H12"/>
-    <mergeCell ref="I9:I12"/>
-    <mergeCell ref="J9:J12"/>
-    <mergeCell ref="G13:G16"/>
-    <mergeCell ref="H13:H16"/>
-    <mergeCell ref="I13:I16"/>
-    <mergeCell ref="J13:J16"/>
-    <mergeCell ref="B2:F2"/>
-    <mergeCell ref="G3:H3"/>
-    <mergeCell ref="I3:J3"/>
-    <mergeCell ref="E9:E12"/>
-    <mergeCell ref="G25:G28"/>
-    <mergeCell ref="H25:H28"/>
-    <mergeCell ref="I25:I28"/>
-    <mergeCell ref="J25:J28"/>
-    <mergeCell ref="G29:G32"/>
-    <mergeCell ref="H29:H32"/>
-    <mergeCell ref="I29:I32"/>
-    <mergeCell ref="J29:J32"/>
-    <mergeCell ref="G17:G20"/>
-    <mergeCell ref="H17:H20"/>
-    <mergeCell ref="I17:I20"/>
-    <mergeCell ref="J17:J20"/>
-    <mergeCell ref="G21:G24"/>
-    <mergeCell ref="H21:H24"/>
-    <mergeCell ref="I21:I24"/>
-    <mergeCell ref="J21:J24"/>
-    <mergeCell ref="G41:G44"/>
-    <mergeCell ref="H41:H44"/>
-    <mergeCell ref="I41:I44"/>
-    <mergeCell ref="J41:J44"/>
-    <mergeCell ref="G45:G48"/>
-    <mergeCell ref="H45:H48"/>
-    <mergeCell ref="I45:I48"/>
-    <mergeCell ref="J45:J48"/>
-    <mergeCell ref="G33:G36"/>
-    <mergeCell ref="H33:H36"/>
-    <mergeCell ref="I33:I36"/>
-    <mergeCell ref="J33:J36"/>
-    <mergeCell ref="G37:G40"/>
-    <mergeCell ref="H37:H40"/>
-    <mergeCell ref="I37:I40"/>
-    <mergeCell ref="J37:J40"/>
-    <mergeCell ref="G57:G60"/>
-    <mergeCell ref="H57:H60"/>
-    <mergeCell ref="I57:I60"/>
-    <mergeCell ref="J57:J60"/>
-    <mergeCell ref="G61:G64"/>
-    <mergeCell ref="H61:H64"/>
-    <mergeCell ref="I61:I64"/>
-    <mergeCell ref="J61:J64"/>
-    <mergeCell ref="G49:G52"/>
-    <mergeCell ref="H49:H52"/>
-    <mergeCell ref="I49:I52"/>
-    <mergeCell ref="J49:J52"/>
-    <mergeCell ref="G53:G56"/>
-    <mergeCell ref="H53:H56"/>
-    <mergeCell ref="I53:I56"/>
-    <mergeCell ref="J53:J56"/>
+    <mergeCell ref="A29:A32"/>
+    <mergeCell ref="B29:B32"/>
+    <mergeCell ref="C29:C32"/>
+    <mergeCell ref="D29:D32"/>
+    <mergeCell ref="E29:E32"/>
+    <mergeCell ref="A25:A28"/>
+    <mergeCell ref="B25:B28"/>
+    <mergeCell ref="C25:C28"/>
+    <mergeCell ref="D25:D28"/>
+    <mergeCell ref="E25:E28"/>
+    <mergeCell ref="A37:A40"/>
+    <mergeCell ref="B37:B40"/>
+    <mergeCell ref="C37:C40"/>
+    <mergeCell ref="D37:D40"/>
+    <mergeCell ref="E37:E40"/>
+    <mergeCell ref="A33:A36"/>
+    <mergeCell ref="B33:B36"/>
+    <mergeCell ref="C33:C36"/>
+    <mergeCell ref="D33:D36"/>
+    <mergeCell ref="E33:E36"/>
+    <mergeCell ref="A45:A48"/>
+    <mergeCell ref="B45:B48"/>
+    <mergeCell ref="C45:C48"/>
+    <mergeCell ref="D45:D48"/>
+    <mergeCell ref="E45:E48"/>
+    <mergeCell ref="A41:A44"/>
+    <mergeCell ref="B41:B44"/>
+    <mergeCell ref="C41:C44"/>
+    <mergeCell ref="E41:E44"/>
+    <mergeCell ref="D41:D44"/>
+    <mergeCell ref="A53:A56"/>
+    <mergeCell ref="B53:B56"/>
+    <mergeCell ref="C53:C56"/>
+    <mergeCell ref="D53:D56"/>
+    <mergeCell ref="E53:E56"/>
+    <mergeCell ref="A49:A52"/>
+    <mergeCell ref="B49:B52"/>
+    <mergeCell ref="C49:C52"/>
+    <mergeCell ref="D49:D52"/>
+    <mergeCell ref="E49:E52"/>
+    <mergeCell ref="A61:A64"/>
+    <mergeCell ref="B61:B64"/>
+    <mergeCell ref="C61:C64"/>
+    <mergeCell ref="D61:D64"/>
+    <mergeCell ref="E61:E64"/>
+    <mergeCell ref="A57:A60"/>
+    <mergeCell ref="B57:B60"/>
+    <mergeCell ref="C57:C60"/>
+    <mergeCell ref="D57:D60"/>
+    <mergeCell ref="E57:E60"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4087,221 +4090,221 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:12" x14ac:dyDescent="0.15">
-      <c r="B2" s="37" t="s">
+      <c r="B2" s="26" t="s">
         <v>89</v>
       </c>
-      <c r="C2" s="38"/>
-      <c r="D2" s="38"/>
-      <c r="E2" s="38"/>
-      <c r="F2" s="39"/>
-      <c r="H2" s="45" t="s">
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="28"/>
+      <c r="H2" s="19" t="s">
         <v>90</v>
       </c>
-      <c r="I2" s="46"/>
-      <c r="J2" s="46"/>
-      <c r="K2" s="46"/>
-      <c r="L2" s="47"/>
+      <c r="I2" s="20"/>
+      <c r="J2" s="20"/>
+      <c r="K2" s="20"/>
+      <c r="L2" s="21"/>
     </row>
     <row r="3" spans="2:12" x14ac:dyDescent="0.15">
-      <c r="B3" s="40"/>
-      <c r="C3" s="40"/>
-      <c r="D3" s="40"/>
-      <c r="E3" s="40"/>
-      <c r="F3" s="40"/>
-      <c r="H3" s="48"/>
-      <c r="I3" s="48"/>
-      <c r="J3" s="48"/>
-      <c r="K3" s="48"/>
-      <c r="L3" s="48"/>
+      <c r="B3" s="13"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
+      <c r="F3" s="13"/>
+      <c r="H3" s="16"/>
+      <c r="I3" s="16"/>
+      <c r="J3" s="16"/>
+      <c r="K3" s="16"/>
+      <c r="L3" s="16"/>
     </row>
     <row r="4" spans="2:12" ht="27" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B4" s="41" t="s">
+      <c r="B4" s="24" t="s">
         <v>75</v>
       </c>
-      <c r="C4" s="42"/>
-      <c r="D4" s="40"/>
-      <c r="E4" s="41" t="s">
+      <c r="C4" s="25"/>
+      <c r="D4" s="13"/>
+      <c r="E4" s="24" t="s">
         <v>76</v>
       </c>
-      <c r="F4" s="42"/>
-      <c r="H4" s="49" t="s">
+      <c r="F4" s="25"/>
+      <c r="H4" s="22" t="s">
         <v>75</v>
       </c>
-      <c r="I4" s="50"/>
-      <c r="J4" s="48"/>
-      <c r="K4" s="49" t="s">
+      <c r="I4" s="23"/>
+      <c r="J4" s="16"/>
+      <c r="K4" s="22" t="s">
         <v>76</v>
       </c>
-      <c r="L4" s="50"/>
+      <c r="L4" s="23"/>
     </row>
     <row r="5" spans="2:12" x14ac:dyDescent="0.15">
-      <c r="B5" s="43" t="s">
-        <v>53</v>
-      </c>
-      <c r="C5" s="43" t="s">
-        <v>54</v>
-      </c>
-      <c r="D5" s="40"/>
-      <c r="E5" s="43" t="s">
-        <v>53</v>
-      </c>
-      <c r="F5" s="43" t="s">
-        <v>54</v>
-      </c>
-      <c r="H5" s="51" t="s">
-        <v>53</v>
-      </c>
-      <c r="I5" s="51" t="s">
-        <v>54</v>
-      </c>
-      <c r="J5" s="48"/>
-      <c r="K5" s="51" t="s">
-        <v>53</v>
-      </c>
-      <c r="L5" s="51" t="s">
+      <c r="B5" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="C5" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="D5" s="13"/>
+      <c r="E5" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="F5" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="H5" s="17" t="s">
+        <v>53</v>
+      </c>
+      <c r="I5" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="J5" s="16"/>
+      <c r="K5" s="17" t="s">
+        <v>53</v>
+      </c>
+      <c r="L5" s="17" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="6" spans="2:12" x14ac:dyDescent="0.15">
-      <c r="B6" s="44">
+      <c r="B6" s="15">
         <f>COUNTIF(Resultados!B$5:B$64,"Ok")/(COUNT('Casos de Regatas y sus Títulos'!A$3:A$17))</f>
         <v>0.8</v>
       </c>
-      <c r="C6" s="44">
+      <c r="C6" s="15">
         <f>COUNTIF(Resultados!B$5:B$64,"Falla")/(COUNT('Casos de Regatas y sus Títulos'!A$3:A$17))</f>
         <v>0.2</v>
       </c>
-      <c r="D6" s="40"/>
-      <c r="E6" s="44">
+      <c r="D6" s="13"/>
+      <c r="E6" s="15">
         <f>COUNTIF(Resultados!C$5:C$64,"Ok")/(COUNT('Casos de Regatas y sus Títulos'!A$3:A$17))</f>
         <v>0.53333333333333333</v>
       </c>
-      <c r="F6" s="44">
+      <c r="F6" s="15">
         <f>COUNTIF(Resultados!C$5:C$64,"Falla")/(COUNT('Casos de Regatas y sus Títulos'!A$3:A$17))</f>
         <v>0.46666666666666667</v>
       </c>
-      <c r="H6" s="52">
+      <c r="H6" s="18">
         <f>COUNTIF(Resultados!G$5:G$64,"Ok")/(COUNT('Casos de Regatas y sus Títulos'!A$3:A$17))</f>
         <v>0.66666666666666663</v>
       </c>
-      <c r="I6" s="52">
+      <c r="I6" s="18">
         <f>COUNTIF(Resultados!G$5:G$64,"Falla")/(COUNT('Casos de Regatas y sus Títulos'!A$3:A$17))</f>
         <v>0.33333333333333331</v>
       </c>
-      <c r="J6" s="48"/>
-      <c r="K6" s="52">
+      <c r="J6" s="16"/>
+      <c r="K6" s="18">
         <f>COUNTIF(Resultados!H$5:H$64,"Ok")/(COUNT('Casos de Regatas y sus Títulos'!A$3:A$17))</f>
         <v>0.53333333333333333</v>
       </c>
-      <c r="L6" s="52">
+      <c r="L6" s="18">
         <f>COUNTIF(Resultados!H$5:H$64,"Falla")/(COUNT('Casos de Regatas y sus Títulos'!A$3:A$17))</f>
         <v>0.46666666666666667</v>
       </c>
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.15">
-      <c r="B7" s="40"/>
-      <c r="C7" s="40"/>
-      <c r="D7" s="40"/>
-      <c r="E7" s="40"/>
-      <c r="F7" s="40"/>
-      <c r="H7" s="48"/>
-      <c r="I7" s="48"/>
-      <c r="J7" s="48"/>
-      <c r="K7" s="48"/>
-      <c r="L7" s="48"/>
+      <c r="B7" s="13"/>
+      <c r="C7" s="13"/>
+      <c r="D7" s="13"/>
+      <c r="E7" s="13"/>
+      <c r="F7" s="13"/>
+      <c r="H7" s="16"/>
+      <c r="I7" s="16"/>
+      <c r="J7" s="16"/>
+      <c r="K7" s="16"/>
+      <c r="L7" s="16"/>
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.15">
-      <c r="B8" s="40"/>
-      <c r="C8" s="40"/>
-      <c r="D8" s="40"/>
-      <c r="E8" s="40"/>
-      <c r="F8" s="40"/>
-      <c r="H8" s="48"/>
-      <c r="I8" s="48"/>
-      <c r="J8" s="48"/>
-      <c r="K8" s="48"/>
-      <c r="L8" s="48"/>
+      <c r="B8" s="13"/>
+      <c r="C8" s="13"/>
+      <c r="D8" s="13"/>
+      <c r="E8" s="13"/>
+      <c r="F8" s="13"/>
+      <c r="H8" s="16"/>
+      <c r="I8" s="16"/>
+      <c r="J8" s="16"/>
+      <c r="K8" s="16"/>
+      <c r="L8" s="16"/>
     </row>
     <row r="9" spans="2:12" ht="28" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B9" s="41" t="s">
+      <c r="B9" s="24" t="s">
         <v>87</v>
       </c>
-      <c r="C9" s="42"/>
-      <c r="D9" s="40"/>
-      <c r="E9" s="41" t="s">
+      <c r="C9" s="25"/>
+      <c r="D9" s="13"/>
+      <c r="E9" s="24" t="s">
         <v>88</v>
       </c>
-      <c r="F9" s="42"/>
-      <c r="H9" s="49" t="s">
+      <c r="F9" s="25"/>
+      <c r="H9" s="22" t="s">
         <v>87</v>
       </c>
-      <c r="I9" s="50"/>
-      <c r="J9" s="48"/>
-      <c r="K9" s="49" t="s">
+      <c r="I9" s="23"/>
+      <c r="J9" s="16"/>
+      <c r="K9" s="22" t="s">
         <v>88</v>
       </c>
-      <c r="L9" s="50"/>
+      <c r="L9" s="23"/>
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.15">
-      <c r="B10" s="43" t="s">
-        <v>53</v>
-      </c>
-      <c r="C10" s="43" t="s">
-        <v>54</v>
-      </c>
-      <c r="D10" s="40"/>
-      <c r="E10" s="43" t="s">
-        <v>53</v>
-      </c>
-      <c r="F10" s="43" t="s">
-        <v>54</v>
-      </c>
-      <c r="H10" s="51" t="s">
-        <v>53</v>
-      </c>
-      <c r="I10" s="51" t="s">
-        <v>54</v>
-      </c>
-      <c r="J10" s="48"/>
-      <c r="K10" s="51" t="s">
-        <v>53</v>
-      </c>
-      <c r="L10" s="51" t="s">
+      <c r="B10" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="C10" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="D10" s="13"/>
+      <c r="E10" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="F10" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="H10" s="17" t="s">
+        <v>53</v>
+      </c>
+      <c r="I10" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="J10" s="16"/>
+      <c r="K10" s="17" t="s">
+        <v>53</v>
+      </c>
+      <c r="L10" s="17" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.15">
-      <c r="B11" s="44">
+      <c r="B11" s="15">
         <f>COUNTIF(Resultados!D$5:D$64,"Ok")/(COUNT('Casos de Regatas y sus Títulos'!A$3:A$17))</f>
         <v>0.46666666666666667</v>
       </c>
-      <c r="C11" s="44">
+      <c r="C11" s="15">
         <f>COUNTIF(Resultados!D$5:D$64,"Falla")/(COUNT('Casos de Regatas y sus Títulos'!A$3:A$17))</f>
         <v>0.53333333333333333</v>
       </c>
-      <c r="D11" s="40"/>
-      <c r="E11" s="44">
+      <c r="D11" s="13"/>
+      <c r="E11" s="15">
         <f>COUNTIF(Resultados!E$5:E$64,"Ok")/(COUNT('Casos de Regatas y sus Títulos'!A$3:A$17))</f>
         <v>0.46666666666666667</v>
       </c>
-      <c r="F11" s="44">
+      <c r="F11" s="15">
         <f>COUNTIF(Resultados!E$5:E$64,"Falla")/(COUNT('Casos de Regatas y sus Títulos'!A$3:A$17))</f>
         <v>0.53333333333333333</v>
       </c>
-      <c r="H11" s="52">
+      <c r="H11" s="18">
         <f>COUNTIF(Resultados!I$5:I$64,"Ok")/(COUNT('Casos de Regatas y sus Títulos'!A$3:A$17))</f>
         <v>0.73333333333333328</v>
       </c>
-      <c r="I11" s="52">
+      <c r="I11" s="18">
         <f>COUNTIF(Resultados!I$5:I$64,"Falla")/(COUNT('Casos de Regatas y sus Títulos'!A$3:A$17))</f>
         <v>0.26666666666666666</v>
       </c>
-      <c r="J11" s="48"/>
-      <c r="K11" s="52">
+      <c r="J11" s="16"/>
+      <c r="K11" s="18">
         <f>COUNTIF(Resultados!J$5:J$64,"Ok")/(COUNT('Casos de Regatas y sus Títulos'!A$3:A$17))</f>
         <v>0.66666666666666663</v>
       </c>
-      <c r="L11" s="52">
+      <c r="L11" s="18">
         <f>COUNTIF(Resultados!J$5:J$64,"Falla")/(COUNT('Casos de Regatas y sus Títulos'!A$3:A$17))</f>
         <v>0.33333333333333331</v>
       </c>
@@ -4311,16 +4314,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="E9:F9"/>
+    <mergeCell ref="B2:F2"/>
     <mergeCell ref="H2:L2"/>
     <mergeCell ref="H4:I4"/>
     <mergeCell ref="K4:L4"/>
     <mergeCell ref="H9:I9"/>
     <mergeCell ref="K9:L9"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="E4:F4"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="E9:F9"/>
-    <mergeCell ref="B2:F2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>